<commit_message>
Release btp_valore_ottobre_2026.xlsx: video YouTube live
</commit_message>
<xml_diff>
--- a/simulatori/btp_valore_ottobre_2026.xlsx
+++ b/simulatori/btp_valore_ottobre_2026.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="172">
   <si>
     <t>Simulatore BTP Valore e BTP Valore Insieme — ottobre 2026</t>
   </si>
@@ -108,7 +108,7 @@
     <t>Tasso cedolare annuo, anno 1</t>
   </si>
   <si>
-    <t>Esempio compatibile con la previsione: scrivi qui i tassi veri, anno per anno</t>
+    <t>Tassi minimi garantiti del comunicato MEF n. 110 del 16/10/2026 (ISIN IT0005735201). A fine collocamento possono solo salire: se salgono, scrivili qui</t>
   </si>
   <si>
     <t>Tasso cedolare annuo, anno 2</t>
@@ -126,13 +126,13 @@
     <t>Valore Insieme: cedola unica annunciata (% del capitale, lorda)</t>
   </si>
   <si>
-    <t>Se vuota, il foglio usa quella equivalente al rendimento del Valore trimestrale</t>
+    <t>22,25% minimo garantito, comunicato MEF n. 110 del 16/10/2026 (ISIN IT0005735227). Se svuoti la cella, il foglio usa la cedola equivalente al Valore trimestrale</t>
   </si>
   <si>
     <t>Rendimento lordo BTP 3,95% feb-2032 su Borsa Italiana, quel giorno</t>
   </si>
   <si>
-    <t>Il nuovo BTP a 5 anni (asta del 29/09/2026). Al 25/09 il riferimento era il BTP giu-2031: 3,99% sul prezzo MOT 96,59</t>
+    <t>BTP 3,95% feb-2032 (IT0005733636): 4,01% lordo su Borsa Italiana il 16/10/2026, prezzo di riferimento 99,90. Al 25/09 il riferimento era il BTP giu-2031: 3,99% sul prezzo MOT 96,59</t>
   </si>
   <si>
     <t>Aliquota imposta titoli di Stato</t>
@@ -375,7 +375,7 @@
     <t>Differenza (positivo = meglio il trimestrale)</t>
   </si>
   <si>
-    <t>Approssimazione: le cedole di ogni anno reinvestite in media a metà anno.</t>
+    <t>Ogni cedola netta trimestrale reinvestita dal giorno in cui la incassi fino alla scadenza, al tasso annuo di B7.</t>
   </si>
   <si>
     <t>Se vendi prima: prezzo dei due gemelli (per 100 di nominale)</t>
@@ -507,13 +507,22 @@
     <t>a 100 in collocamento</t>
   </si>
   <si>
-    <t>Previsione mia, non un dato</t>
+    <t>Previsione mia del 25/09, non un dato</t>
+  </si>
+  <si>
+    <t>Nuovo BTP Valore, tassi minimi del 16/10</t>
+  </si>
+  <si>
+    <t>a 100 in collocamento, 19-23/10/2026</t>
+  </si>
+  <si>
+    <t>Calcolo mio sul comunicato MEF n. 110 del 16/10/2026</t>
   </si>
   <si>
     <t>Inflazione di pareggio: nuovo Valore contro BTP Italia Sì comprato oggi a ~100</t>
   </si>
   <si>
-    <t>Rendimento lordo del nuovo Valore</t>
+    <t>Rendimento lordo del nuovo Valore (dal foglio 1)</t>
   </si>
   <si>
     <t>Tasso reale del BTP Italia Sì</t>
@@ -1185,12 +1194,12 @@
       <c r="D4" s="21"/>
       <c r="E4" s="21"/>
     </row>
-    <row r="5" spans="1:5" ht="45" customHeight="1">
+    <row r="5" spans="1:5" ht="90" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B5" s="6">
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>29</v>
@@ -1203,7 +1212,7 @@
         <v>30</v>
       </c>
       <c r="B6" s="6">
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1211,7 +1220,7 @@
         <v>31</v>
       </c>
       <c r="B7" s="6">
-        <v>3.7999999999999999E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1219,7 +1228,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="6">
-        <v>4.2999999999999997E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1227,26 +1236,28 @@
         <v>33</v>
       </c>
       <c r="B9" s="6">
-        <v>4.2999999999999997E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="45" customHeight="1">
+        <v>4.7E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="90" customHeight="1">
       <c r="A10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="6"/>
+      <c r="B10" s="6">
+        <v>0.2225</v>
+      </c>
       <c r="C10" s="24" t="s">
         <v>35</v>
       </c>
       <c r="D10" s="21"/>
       <c r="E10" s="21"/>
     </row>
-    <row r="11" spans="1:5" ht="75" customHeight="1">
+    <row r="11" spans="1:5" ht="105" customHeight="1">
       <c r="A11" s="5" t="s">
         <v>36</v>
       </c>
       <c r="B11" s="6">
-        <v>0.04</v>
+        <v>4.0099999999999997E-2</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>37</v>
@@ -1296,11 +1307,11 @@
       </c>
       <c r="B17" s="10">
         <f>(1+IRR(D40:D60))^4-1</f>
-        <v>4.048226182085557E-2</v>
+        <v>4.102488434039131E-2</v>
       </c>
       <c r="C17" s="10">
         <f>IF(ISBLANK(B10),B17,(1+B10)^(1/5)-1)</f>
-        <v>4.048226182085557E-2</v>
+        <v>4.0997708595530424E-2</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1309,11 +1320,11 @@
       </c>
       <c r="B18" s="10">
         <f>(1+IRR(E40:E60))^4-1</f>
-        <v>3.5369006773171785E-2</v>
+        <v>3.5850134757430929E-2</v>
       </c>
       <c r="C18" s="10">
         <f>(1+C19*(1-B12))^(1/5)-1</f>
-        <v>3.5758011521765276E-2</v>
+        <v>3.6217360208301352E-2</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1322,11 +1333,11 @@
       </c>
       <c r="B19" s="10">
         <f>SUM(B5:B9)</f>
-        <v>0.19999999999999996</v>
+        <v>0.20300000000000001</v>
       </c>
       <c r="C19" s="10">
         <f>IF(ISBLANK(B10),(1+B17)^5-1,B10)</f>
-        <v>0.2194764103787934</v>
+        <v>0.2225</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1335,11 +1346,11 @@
       </c>
       <c r="B20" s="11">
         <f>B19*B13</f>
-        <v>1999.9999999999995</v>
+        <v>2030.0000000000002</v>
       </c>
       <c r="C20" s="11">
         <f>C19*B13</f>
-        <v>2194.7641037879339</v>
+        <v>2225</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1348,11 +1359,11 @@
       </c>
       <c r="B21" s="11">
         <f>B20*(1-B12)</f>
-        <v>1749.9999999999995</v>
+        <v>1776.2500000000002</v>
       </c>
       <c r="C21" s="11">
         <f>C20*(1-B12)</f>
-        <v>1920.4185908144423</v>
+        <v>1946.875</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1361,7 +1372,7 @@
       </c>
       <c r="B22" s="10">
         <f>AVERAGE(B5:B9)</f>
-        <v>3.9999999999999994E-2</v>
+        <v>4.0600000000000004E-2</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1370,11 +1381,11 @@
       </c>
       <c r="B23" s="12">
         <f>(B17-B11)*100</f>
-        <v>4.8226182085556873E-2</v>
+        <v>9.2488434039131318E-2</v>
       </c>
       <c r="C23" s="12">
         <f>(C17-B11)*100</f>
-        <v>4.8226182085556873E-2</v>
+        <v>8.9770859553042759E-2</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1459,15 +1470,15 @@
       </c>
       <c r="C41" s="10">
         <f t="shared" ref="C41:C60" si="1">INDEX($B$5:$B$9,B41)</f>
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="D41" s="15">
         <f t="shared" ref="D41:D59" si="2">100*C41/4</f>
-        <v>0.95</v>
+        <v>0.92499999999999993</v>
       </c>
       <c r="E41" s="15">
         <f t="shared" ref="E41:E59" si="3">100*C41/4*(1-$B$12)</f>
-        <v>0.83124999999999993</v>
+        <v>0.80937499999999996</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -1480,15 +1491,15 @@
       </c>
       <c r="C42" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="D42" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>0.92499999999999993</v>
       </c>
       <c r="E42" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.80937499999999996</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -1501,15 +1512,15 @@
       </c>
       <c r="C43" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="D43" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>0.92499999999999993</v>
       </c>
       <c r="E43" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.80937499999999996</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -1522,15 +1533,15 @@
       </c>
       <c r="C44" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="D44" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>0.92499999999999993</v>
       </c>
       <c r="E44" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.80937499999999996</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -1543,15 +1554,15 @@
       </c>
       <c r="C45" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="D45" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>0.92499999999999993</v>
       </c>
       <c r="E45" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.80937499999999996</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -1564,15 +1575,15 @@
       </c>
       <c r="C46" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="D46" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>0.92499999999999993</v>
       </c>
       <c r="E46" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.80937499999999996</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -1585,15 +1596,15 @@
       </c>
       <c r="C47" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="D47" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>0.92499999999999993</v>
       </c>
       <c r="E47" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.80937499999999996</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -1606,15 +1617,15 @@
       </c>
       <c r="C48" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
       <c r="D48" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>0.92499999999999993</v>
       </c>
       <c r="E48" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.80937499999999996</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -1627,15 +1638,15 @@
       </c>
       <c r="C49" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="D49" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>1.0250000000000001</v>
       </c>
       <c r="E49" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.89687500000000009</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -1648,15 +1659,15 @@
       </c>
       <c r="C50" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="D50" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>1.0250000000000001</v>
       </c>
       <c r="E50" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.89687500000000009</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -1669,15 +1680,15 @@
       </c>
       <c r="C51" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="D51" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>1.0250000000000001</v>
       </c>
       <c r="E51" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.89687500000000009</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -1690,15 +1701,15 @@
       </c>
       <c r="C52" s="10">
         <f t="shared" si="1"/>
-        <v>3.7999999999999999E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="D52" s="15">
         <f t="shared" si="2"/>
-        <v>0.95</v>
+        <v>1.0250000000000001</v>
       </c>
       <c r="E52" s="15">
         <f t="shared" si="3"/>
-        <v>0.83124999999999993</v>
+        <v>0.89687500000000009</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -1711,15 +1722,15 @@
       </c>
       <c r="C53" s="10">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="D53" s="15">
         <f t="shared" si="2"/>
-        <v>1.075</v>
+        <v>1.0250000000000001</v>
       </c>
       <c r="E53" s="15">
         <f t="shared" si="3"/>
-        <v>0.94062499999999993</v>
+        <v>0.89687500000000009</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -1732,15 +1743,15 @@
       </c>
       <c r="C54" s="10">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="D54" s="15">
         <f t="shared" si="2"/>
-        <v>1.075</v>
+        <v>1.0250000000000001</v>
       </c>
       <c r="E54" s="15">
         <f t="shared" si="3"/>
-        <v>0.94062499999999993</v>
+        <v>0.89687500000000009</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -1753,15 +1764,15 @@
       </c>
       <c r="C55" s="10">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="D55" s="15">
         <f t="shared" si="2"/>
-        <v>1.075</v>
+        <v>1.0250000000000001</v>
       </c>
       <c r="E55" s="15">
         <f t="shared" si="3"/>
-        <v>0.94062499999999993</v>
+        <v>0.89687500000000009</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -1774,15 +1785,15 @@
       </c>
       <c r="C56" s="10">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="D56" s="15">
         <f t="shared" si="2"/>
-        <v>1.075</v>
+        <v>1.0250000000000001</v>
       </c>
       <c r="E56" s="15">
         <f t="shared" si="3"/>
-        <v>0.94062499999999993</v>
+        <v>0.89687500000000009</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -1795,15 +1806,15 @@
       </c>
       <c r="C57" s="10">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="D57" s="15">
         <f t="shared" si="2"/>
-        <v>1.075</v>
+        <v>1.175</v>
       </c>
       <c r="E57" s="15">
         <f t="shared" si="3"/>
-        <v>0.94062499999999993</v>
+        <v>1.028125</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -1816,15 +1827,15 @@
       </c>
       <c r="C58" s="10">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="D58" s="15">
         <f t="shared" si="2"/>
-        <v>1.075</v>
+        <v>1.175</v>
       </c>
       <c r="E58" s="15">
         <f t="shared" si="3"/>
-        <v>0.94062499999999993</v>
+        <v>1.028125</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -1837,15 +1848,15 @@
       </c>
       <c r="C59" s="10">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="D59" s="15">
         <f t="shared" si="2"/>
-        <v>1.075</v>
+        <v>1.175</v>
       </c>
       <c r="E59" s="15">
         <f t="shared" si="3"/>
-        <v>0.94062499999999993</v>
+        <v>1.028125</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -1858,15 +1869,15 @@
       </c>
       <c r="C60" s="10">
         <f t="shared" si="1"/>
-        <v>4.2999999999999997E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="D60" s="15">
         <f>100*C60/4 + 100</f>
-        <v>101.075</v>
+        <v>101.175</v>
       </c>
       <c r="E60" s="15">
         <f>100*C60/4*(1-$B$12) + 100</f>
-        <v>100.940625</v>
+        <v>101.028125</v>
       </c>
     </row>
   </sheetData>
@@ -2293,7 +2304,7 @@
       </c>
       <c r="B5" s="10">
         <f>'1 - Il 16 ottobre'!B17</f>
-        <v>4.048226182085557E-2</v>
+        <v>4.102488434039131E-2</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -2309,7 +2320,7 @@
         <v>104</v>
       </c>
       <c r="B7" s="6">
-        <v>3.5000000000000003E-2</v>
+        <v>3.5799999999999998E-2</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>105</v>
@@ -2348,11 +2359,11 @@
       </c>
       <c r="B10" s="11">
         <f>$B$4*INDEX('1 - Il 16 ottobre'!$B$5:$B$9,A10)</f>
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C10" s="11">
         <f>B10*(1-'1 - Il 16 ottobre'!$B$12)</f>
-        <v>332.5</v>
+        <v>323.75</v>
       </c>
       <c r="D10" s="11">
         <f>$B$4*$B$6</f>
@@ -2364,11 +2375,11 @@
       </c>
       <c r="F10" s="11">
         <f>$B$4*(1+'1 - Il 16 ottobre'!$C$17)^A10</f>
-        <v>10404.822618208556</v>
+        <v>10409.977085955305</v>
       </c>
       <c r="G10" s="11">
         <f>F10*$B$6</f>
-        <v>20.809645236417115</v>
+        <v>20.819954171910609</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -2377,11 +2388,11 @@
       </c>
       <c r="B11" s="11">
         <f>$B$4*INDEX('1 - Il 16 ottobre'!$B$5:$B$9,A11)</f>
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C11" s="11">
         <f>B11*(1-'1 - Il 16 ottobre'!$B$12)</f>
-        <v>332.5</v>
+        <v>323.75</v>
       </c>
       <c r="D11" s="11">
         <f>$B$4*$B$6</f>
@@ -2393,11 +2404,11 @@
       </c>
       <c r="F11" s="11">
         <f>$B$4*(1+'1 - Il 16 ottobre'!$C$17)^A11</f>
-        <v>10826.033371638436</v>
+        <v>10836.762293011448</v>
       </c>
       <c r="G11" s="11">
         <f>F11*$B$6</f>
-        <v>21.652066743276873</v>
+        <v>21.673524586022896</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2406,11 +2417,11 @@
       </c>
       <c r="B12" s="11">
         <f>$B$4*INDEX('1 - Il 16 ottobre'!$B$5:$B$9,A12)</f>
-        <v>380</v>
+        <v>410</v>
       </c>
       <c r="C12" s="11">
         <f>B12*(1-'1 - Il 16 ottobre'!$B$12)</f>
-        <v>332.5</v>
+        <v>358.75</v>
       </c>
       <c r="D12" s="11">
         <f>$B$4*$B$6</f>
@@ -2422,11 +2433,11 @@
       </c>
       <c r="F12" s="11">
         <f>$B$4*(1+'1 - Il 16 ottobre'!$C$17)^A12</f>
-        <v>11264.295689070423</v>
+        <v>11281.044715619364</v>
       </c>
       <c r="G12" s="11">
         <f>F12*$B$6</f>
-        <v>22.528591378140845</v>
+        <v>22.562089431238729</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2435,11 +2446,11 @@
       </c>
       <c r="B13" s="11">
         <f>$B$4*INDEX('1 - Il 16 ottobre'!$B$5:$B$9,A13)</f>
-        <v>429.99999999999994</v>
+        <v>410</v>
       </c>
       <c r="C13" s="11">
         <f>B13*(1-'1 - Il 16 ottobre'!$B$12)</f>
-        <v>376.24999999999994</v>
+        <v>358.75</v>
       </c>
       <c r="D13" s="11">
         <f>$B$4*$B$6</f>
@@ -2451,11 +2462,11 @@
       </c>
       <c r="F13" s="11">
         <f>$B$4*(1+'1 - Il 16 ottobre'!$C$17)^A13</f>
-        <v>11720.299856382906</v>
+        <v>11743.541699523474</v>
       </c>
       <c r="G13" s="11">
         <f>F13*$B$6</f>
-        <v>23.440599712765813</v>
+        <v>23.487083399046949</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2464,11 +2475,11 @@
       </c>
       <c r="B14" s="11">
         <f>$B$4*INDEX('1 - Il 16 ottobre'!$B$5:$B$9,A14)</f>
-        <v>429.99999999999994</v>
+        <v>470</v>
       </c>
       <c r="C14" s="11">
         <f>B14*(1-'1 - Il 16 ottobre'!$B$12)</f>
-        <v>376.24999999999994</v>
+        <v>411.25</v>
       </c>
       <c r="D14" s="11">
         <f>$B$4*$B$6</f>
@@ -2476,15 +2487,15 @@
       </c>
       <c r="E14" s="11">
         <f>$B$4*'1 - Il 16 ottobre'!$C$19</f>
-        <v>2194.7641037879339</v>
+        <v>2225</v>
       </c>
       <c r="F14" s="11">
         <f>$B$4*(1+'1 - Il 16 ottobre'!$C$17)^A14</f>
-        <v>12194.764103787935</v>
+        <v>12224.999999999996</v>
       </c>
       <c r="G14" s="11">
         <f>F14*$B$6</f>
-        <v>24.389528207575871</v>
+        <v>24.449999999999992</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2493,11 +2504,11 @@
       </c>
       <c r="B15" s="11">
         <f>SUM(B10:B14)</f>
-        <v>2000</v>
+        <v>2030</v>
       </c>
       <c r="C15" s="11">
         <f>SUM(C10:C14)</f>
-        <v>1750</v>
+        <v>1776.25</v>
       </c>
       <c r="D15" s="11">
         <f>SUM(D10:D14)</f>
@@ -2505,11 +2516,11 @@
       </c>
       <c r="E15" s="11">
         <f>SUM(E10:E14)</f>
-        <v>2194.7641037879339</v>
+        <v>2225</v>
       </c>
       <c r="G15" s="11">
         <f>SUM(G10:G14)</f>
-        <v>112.82043127817653</v>
+        <v>112.99265158821918</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="45" customHeight="1">
@@ -2539,8 +2550,8 @@
         <v>115</v>
       </c>
       <c r="B19" s="11">
-        <f>B4+SUMPRODUCT(C10:C14,(1+B7)^(5-A10:A14+0.5))</f>
-        <v>11904.530300396927</v>
+        <f>B4+B4/100*SUMPRODUCT('1 - Il 16 ottobre'!E41:E60-('1 - Il 16 ottobre'!A41:A60=20)*100,(1+B7)^((20-'1 - Il 16 ottobre'!A41:A60)/4))</f>
+        <v>11925.503463267942</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -2549,7 +2560,7 @@
       </c>
       <c r="B20" s="11">
         <f>B4+B4*'1 - Il 16 ottobre'!C19*(1-'1 - Il 16 ottobre'!B12)</f>
-        <v>11920.418590814443</v>
+        <v>11946.875</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -2558,7 +2569,7 @@
       </c>
       <c r="B21" s="11">
         <f>B19-B20</f>
-        <v>-15.888290417515236</v>
+        <v>-21.371536732058303</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="30" customHeight="1">
@@ -2625,7 +2636,7 @@
       </c>
       <c r="B4" s="10">
         <f>'1 - Il 16 ottobre'!B17</f>
-        <v>4.048226182085557E-2</v>
+        <v>4.102488434039131E-2</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="32.1" customHeight="1">
@@ -2654,15 +2665,15 @@
       </c>
       <c r="C7" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A7)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B7/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A7)/4))</f>
-        <v>104.51921506130023</v>
+        <v>104.51926846460589</v>
       </c>
       <c r="D7" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B7/100))^(5-A7)</f>
-        <v>104.94718679107881</v>
+        <v>104.93083554666183</v>
       </c>
       <c r="E7" s="12">
         <f t="shared" ref="E7:E31" si="0">D7-C7</f>
-        <v>0.42797172977857656</v>
+        <v>0.41156708205593873</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -2674,15 +2685,15 @@
       </c>
       <c r="C8" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A8)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B8/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A8)/4))</f>
-        <v>102.22775449876423</v>
+        <v>102.22780306669014</v>
       </c>
       <c r="D8" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B8/100))^(5-A8)</f>
-        <v>102.43776286149637</v>
+        <v>102.42310402939864</v>
       </c>
       <c r="E8" s="12">
         <f t="shared" si="0"/>
-        <v>0.21000836273213963</v>
+        <v>0.19530096270850095</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2694,15 +2705,15 @@
       </c>
       <c r="C9" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A9)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B9/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A9)/4))</f>
-        <v>99.999999999998238</v>
+        <v>99.999999999998508</v>
       </c>
       <c r="D9" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B9/100))^(5-A9)</f>
-        <v>100</v>
+        <v>99.986948282182297</v>
       </c>
       <c r="E9" s="12">
         <f t="shared" si="0"/>
-        <v>1.7621459846850485E-12</v>
+        <v>-1.3051717816210839E-2</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2714,15 +2725,15 @@
       </c>
       <c r="C10" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A10)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B10/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A10)/4))</f>
-        <v>97.833868024363227</v>
+        <v>97.833778540476914</v>
       </c>
       <c r="D10" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B10/100))^(5-A10)</f>
-        <v>97.631522056030093</v>
+        <v>97.619996202127368</v>
       </c>
       <c r="E10" s="12">
         <f t="shared" si="0"/>
-        <v>-0.2023459683331339</v>
+        <v>-0.21378233834954585</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -2734,15 +2745,15 @@
       </c>
       <c r="C11" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A11)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B11/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A11)/4))</f>
-        <v>95.72735295144237</v>
+        <v>95.727135730318295</v>
       </c>
       <c r="D11" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B11/100))^(5-A11)</f>
-        <v>95.330042498217978</v>
+        <v>95.319965107128539</v>
       </c>
       <c r="E11" s="12">
         <f t="shared" si="0"/>
-        <v>-0.39731045322439229</v>
+        <v>-0.4071706231897565</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2754,15 +2765,15 @@
       </c>
       <c r="C12" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A12)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B12/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A12)/4))</f>
-        <v>103.86203163882243</v>
+        <v>104.01919365486289</v>
       </c>
       <c r="D12" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B12/100))^(5-A12)</f>
-        <v>108.1462144162067</v>
+        <v>108.18630258323762</v>
       </c>
       <c r="E12" s="12">
         <f t="shared" si="0"/>
-        <v>4.2841827773842738</v>
+        <v>4.1671089283747307</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2774,15 +2785,15 @@
       </c>
       <c r="C13" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A13)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B13/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A13)/4))</f>
-        <v>102.00483150298921</v>
+        <v>102.16093185720858</v>
       </c>
       <c r="D13" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B13/100))^(5-A13)</f>
-        <v>106.0724863836907</v>
+        <v>106.11288450584161</v>
       </c>
       <c r="E13" s="12">
         <f t="shared" si="0"/>
-        <v>4.0676548807014967</v>
+        <v>3.951952648633025</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2794,15 +2805,15 @@
       </c>
       <c r="C14" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A14)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B14/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A14)/4))</f>
-        <v>100.19101587863912</v>
+        <v>100.34604318286296</v>
       </c>
       <c r="D14" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B14/100))^(5-A14)</f>
-        <v>104.04822618208556</v>
+        <v>104.08890127100751</v>
       </c>
       <c r="E14" s="12">
         <f t="shared" si="0"/>
-        <v>3.8572103034464362</v>
+        <v>3.7428580881445583</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2814,15 +2825,15 @@
       </c>
       <c r="C15" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A15)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B15/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A15)/4))</f>
-        <v>98.419361950616576</v>
+        <v>98.573305979120775</v>
       </c>
       <c r="D15" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B15/100))^(5-A15)</f>
-        <v>102.07202450415107</v>
+        <v>102.1129452366397</v>
       </c>
       <c r="E15" s="12">
         <f t="shared" si="0"/>
-        <v>3.6526625535344976</v>
+        <v>3.5396392575189282</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2834,15 +2845,15 @@
       </c>
       <c r="C16" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A16)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B16/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A16)/4))</f>
-        <v>96.688687087985969</v>
+        <v>96.841538714243669</v>
       </c>
       <c r="D16" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B16/100))^(5-A16)</f>
-        <v>100.1425186630063</v>
+        <v>100.1836553020499</v>
       </c>
       <c r="E16" s="12">
         <f t="shared" si="0"/>
-        <v>3.453831575020331</v>
+        <v>3.3421165878062311</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2854,15 +2865,15 @@
       </c>
       <c r="C17" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A17)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B17/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A17)/4))</f>
-        <v>103.18481577919634</v>
+        <v>103.50360408198608</v>
       </c>
       <c r="D17" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B17/100))^(5-A17)</f>
-        <v>111.44275563897588</v>
+        <v>111.54277010809716</v>
       </c>
       <c r="E17" s="12">
         <f t="shared" si="0"/>
-        <v>8.2579398597795404</v>
+        <v>8.0391660261110758</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2874,15 +2885,15 @@
       </c>
       <c r="C18" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A18)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B18/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A18)/4))</f>
-        <v>101.77399869511223</v>
+        <v>102.09165162013976</v>
       </c>
       <c r="D18" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B18/100))^(5-A18)</f>
-        <v>109.83617811754598</v>
+        <v>109.93558889718986</v>
       </c>
       <c r="E18" s="12">
         <f t="shared" si="0"/>
-        <v>8.0621794224337577</v>
+        <v>7.8439372770501024</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2894,15 +2905,15 @@
       </c>
       <c r="C19" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A19)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B19/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A19)/4))</f>
-        <v>100.38976451209106</v>
+        <v>100.70628274728119</v>
       </c>
       <c r="D19" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B19/100))^(5-A19)</f>
-        <v>108.26033371638434</v>
+        <v>108.359136406769</v>
       </c>
       <c r="E19" s="12">
         <f t="shared" si="0"/>
-        <v>7.8705692042932753</v>
+        <v>7.6528536594878034</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2914,15 +2925,15 @@
       </c>
       <c r="C20" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A20)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B20/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A20)/4))</f>
-        <v>99.031485464918305</v>
+        <v>99.346870082594762</v>
       </c>
       <c r="D20" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B20/100))^(5-A20)</f>
-        <v>106.71449104723365</v>
+        <v>106.81268173081273</v>
       </c>
       <c r="E20" s="12">
         <f t="shared" si="0"/>
-        <v>7.6830055823153458</v>
+        <v>7.4658116482179651</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -2934,15 +2945,15 @@
       </c>
       <c r="C21" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A21)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B21/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A21)/4))</f>
-        <v>97.698551546107865</v>
+        <v>98.012803981532414</v>
       </c>
       <c r="D21" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B21/100))^(5-A21)</f>
-        <v>105.1979395095521</v>
+        <v>105.29551472663464</v>
       </c>
       <c r="E21" s="12">
         <f t="shared" si="0"/>
-        <v>7.4993879634442351</v>
+        <v>7.2827107451022215</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2954,15 +2965,15 @@
       </c>
       <c r="C22" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A22)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B22/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A22)/4))</f>
-        <v>102.48695684842791</v>
+        <v>102.56739429141123</v>
       </c>
       <c r="D22" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B22/100))^(5-A22)</f>
-        <v>114.83978289440078</v>
+        <v>115.00337164970773</v>
       </c>
       <c r="E22" s="12">
         <f t="shared" si="0"/>
-        <v>12.352826045972876</v>
+        <v>12.435977358296498</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -2974,15 +2985,15 @@
       </c>
       <c r="C23" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A23)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B23/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A23)/4))</f>
-        <v>101.53497541710929</v>
+        <v>101.61451167958873</v>
       </c>
       <c r="D23" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B23/100))^(5-A23)</f>
-        <v>113.73341414691488</v>
+        <v>113.89600577210395</v>
       </c>
       <c r="E23" s="12">
         <f t="shared" si="0"/>
-        <v>12.198438729805588</v>
+        <v>12.281494092515217</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -2994,15 +3005,15 @@
       </c>
       <c r="C24" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A24)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B24/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A24)/4))</f>
-        <v>100.59655893975896</v>
+        <v>100.67519890884834</v>
       </c>
       <c r="D24" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B24/100))^(5-A24)</f>
-        <v>112.64295689070421</v>
+        <v>112.80455744508139</v>
       </c>
       <c r="E24" s="12">
         <f t="shared" si="0"/>
-        <v>12.046397950945249</v>
+        <v>12.129358536233042</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -3014,15 +3025,15 @@
       </c>
       <c r="C25" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A25)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B25/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A25)/4))</f>
-        <v>99.67144974116421</v>
+        <v>99.749198367891822</v>
       </c>
       <c r="D25" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B25/100))^(5-A25)</f>
-        <v>111.56810746912328</v>
+        <v>111.72872305356042</v>
       </c>
       <c r="E25" s="12">
         <f t="shared" si="0"/>
-        <v>11.896657727959067</v>
+        <v>11.979524685668594</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -3034,15 +3045,15 @@
       </c>
       <c r="C26" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A26)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B26/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A26)/4))</f>
-        <v>98.75939624620824</v>
+        <v>98.836258540378537</v>
       </c>
       <c r="D26" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B26/100))^(5-A26)</f>
-        <v>110.50856943488782</v>
+        <v>110.66820618712313</v>
       </c>
       <c r="E26" s="12">
         <f t="shared" si="0"/>
-        <v>11.749173188679578</v>
+        <v>11.831947646744595</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -3054,15 +3065,15 @@
       </c>
       <c r="C27" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A27)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B27/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A27)/4))</f>
-        <v>101.26214592779583</v>
+        <v>101.60213870036546</v>
       </c>
       <c r="D27" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B27/100))^(5-A27)</f>
-        <v>118.34035922403811</v>
+        <v>118.57133795389494</v>
       </c>
       <c r="E27" s="12">
         <f t="shared" si="0"/>
-        <v>17.078213296242282</v>
+        <v>16.969199253529482</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -3074,15 +3085,15 @@
       </c>
       <c r="C28" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A28)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B28/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A28)/4))</f>
-        <v>100.7808664543831</v>
+        <v>101.12018282786514</v>
       </c>
       <c r="D28" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B28/100))^(5-A28)</f>
-        <v>117.76893292545553</v>
+        <v>117.99909620687654</v>
       </c>
       <c r="E28" s="12">
         <f t="shared" si="0"/>
-        <v>16.988066471072429</v>
+        <v>16.878913379011408</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -3094,15 +3105,15 @@
       </c>
       <c r="C29" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A29)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B29/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A29)/4))</f>
-        <v>100.30419720208494</v>
+        <v>100.64283985953895</v>
       </c>
       <c r="D29" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B29/100))^(5-A29)</f>
-        <v>117.20299856382906</v>
+        <v>117.43235136733487</v>
       </c>
       <c r="E29" s="12">
         <f t="shared" si="0"/>
-        <v>16.89880136174412</v>
+        <v>16.789511507795922</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -3114,15 +3125,15 @@
       </c>
       <c r="C30" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A30)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B30/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A30)/4))</f>
-        <v>99.832072135681258</v>
+        <v>100.17004376598655</v>
       </c>
       <c r="D30" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B30/100))^(5-A30)</f>
-        <v>116.64247734389127</v>
+        <v>116.87102460960013</v>
       </c>
       <c r="E30" s="12">
         <f t="shared" si="0"/>
-        <v>16.810405208210014</v>
+        <v>16.700980843613578</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -3134,15 +3145,15 @@
       </c>
       <c r="C31" s="15">
         <f>SUMPRODUCT(('1 - Il 16 ottobre'!$A$41:$A$60&gt;4*A31)*'1 - Il 16 ottobre'!$D$41:$D$60/(1+($B$4+B31/100))^(('1 - Il 16 ottobre'!$A$41:$A$60-4*A31)/4))</f>
-        <v>99.364426475872406</v>
+        <v>99.701729772849347</v>
       </c>
       <c r="D31" s="15">
         <f>100*(1+'1 - Il 16 ottobre'!$C$19)/(1+($B$4+B31/100))^(5-A31)</f>
-        <v>116.08729197054802</v>
+        <v>116.31503860797967</v>
       </c>
       <c r="E31" s="12">
         <f t="shared" si="0"/>
-        <v>16.722865494675617</v>
+        <v>16.613308835130326</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="150" customHeight="1">
@@ -3169,7 +3180,7 @@
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="40.140625" customWidth="1"/>
+    <col min="1" max="1" width="55.7109375" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="13.140625" customWidth="1"/>
@@ -3375,9 +3386,29 @@
         <v>162</v>
       </c>
     </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="C13" s="6">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="D13" s="6">
+        <v>3.5900000000000001E-2</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>165</v>
+      </c>
+    </row>
     <row r="14" spans="1:6">
       <c r="A14" s="23" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="21"/>
@@ -3387,15 +3418,16 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="B15" s="6">
-        <v>4.0500000000000001E-2</v>
+        <v>167</v>
+      </c>
+      <c r="B15" s="10">
+        <f>'1 - Il 16 ottobre'!B17</f>
+        <v>4.102488434039131E-2</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="5" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B16" s="6">
         <v>1.6E-2</v>
@@ -3403,16 +3435,16 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B17" s="10">
         <f>(1+B15)/(1+B16)-1</f>
-        <v>2.4114173228346525E-2</v>
+        <v>2.4630791673613484E-2</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="30" customHeight="1">
       <c r="A18" s="24" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B18" s="21"/>
       <c r="C18" s="21"/>
@@ -3422,7 +3454,7 @@
     </row>
     <row r="20" spans="1:6" ht="60" customHeight="1">
       <c r="A20" s="24" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B20" s="21"/>
       <c r="C20" s="21"/>

</xml_diff>